<commit_message>
Add 7 new baselines: PromptArmor, RENNERVATE, SkillScan, Attention Tracker, cisco, Wen2025, MASB pipeline
</commit_message>
<xml_diff>
--- a/related_work.xlsx
+++ b/related_work.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Related Work" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Related Work" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Related Work'!$A$1:$F$32</definedName>
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1546,6 +1546,230 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Static Analysis</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SkillScan: Static + LLM Semantic Classification</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2601.10338</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>arXiv 2026</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>多层次静态分析+LLM语义分类管线，代表"混合筛查"家族。开源工具包和数据集，复现成本低</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>文本侧方法，不读hidden state——与我们互补。可作为surface-text对比基线</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Static Analysis</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PromptArmor: Universal Prompt Injection Defense</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2507.15219</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>arXiv 2025</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Dawn Song组，最强文本侧通用IPI防御，代表"prompt清洗/过滤"家族</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>纯文本清洗。作为文本侧最强基线对比</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Hidden-State Detection</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>RENNERVATE: Attention-Based Detection</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2512.08417</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>arXiv 2025</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>注意力/隐状态检测器，RouteGuard表4/5中最强竞争者(BIPIA F1 0.7815 vs RG 0.8537)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>最直接内部信号竞争者——必须在实验表中对比</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hidden-State Detection</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Attention Tracker: Attention Routing for Injection Detection</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2411.00348</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>arXiv 2024, IBM</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>注意力路由信号做注入检测的先驱。内部信号路线的经典参照点</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>早期注意力方法——可与RouteGuard一同作为内部信号基线</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sandbox / Dynamic</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Malicious Agent Skills in the Wild (MASB pipeline)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.06547</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>arXiv 2026</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>静态模式匹配+动态行为验证，代表"行为确认"家族。157个确认恶意skill+protectskills仓库</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>数据基座来源。其157恶意skill是我们的MASB 75K数据源</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Mechanistic / Rep</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Wen et al. 2025: Instruction Detection via Representations</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ACL Findings</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ACL 2025 Findings</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>基于表征的指令检测。如果你的方法涉及hidden-state对齐，这是最贴的先验工作</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>表征对齐方法论参考</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Static Analysis</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>cisco-ai-skill-scanner</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://github.com/cisco-ai/skill-scanner</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>工业界官方工具，无论文但可直接运行。加一个"真实部署扫描器"基线提升可信度</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>零成本工业基线。直接可运行</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>